<commit_message>
Materi Kuliah Basis Data
</commit_message>
<xml_diff>
--- a/Studi Kasus - Tabungan Bank/Lampiran ERD - Tabungan.xlsx
+++ b/Studi Kasus - Tabungan Bank/Lampiran ERD - Tabungan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Materi Kuliah - Basis Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Meteri Kuliah Basis Data\Studi Kasus - Tabungan Bank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5EC20B0-A9BD-42AF-A443-356EBF16AD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0F3E2E-1806-4589-BAD9-AF39C85A60A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A3570CAD-EB3C-4E13-A541-BB5C9CD63881}"/>
   </bookViews>

</xml_diff>